<commit_message>
accises: onglet Mai-26 AC4 Tea Tree SA — 11 lignes (9 KF + 2 D&B), 614,7 kg, 434,15 EUR
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Accises/AC4_Tea_Tree_SA_Q126_updated v2.xlsx
+++ b/Accises/AC4_Tea_Tree_SA_Q126_updated v2.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DEC25" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q126" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Avril-26" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mai-26" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -25,9 +26,9 @@
     <numFmt numFmtId="167" formatCode="dd/mm/yy"/>
     <numFmt numFmtId="168" formatCode="DD/MM/YYYY"/>
     <numFmt numFmtId="169" formatCode="#,##0.00 €"/>
-    <numFmt numFmtId="170" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="171" formatCode="dd-mm-yyyy"/>
-    <numFmt numFmtId="172" formatCode="#,##0.000000"/>
+    <numFmt numFmtId="170" formatCode="dd-mm-yyyy"/>
+    <numFmt numFmtId="171" formatCode="#,##0.000000"/>
+    <numFmt numFmtId="172" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -320,7 +321,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="115">
+  <cellXfs count="118">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -627,9 +628,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="171" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -56935,32 +56939,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="0" t="inlineStr">
         <is>
           <t>Avril26</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="0" t="inlineStr">
         <is>
           <t>Avril26</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="0" t="inlineStr">
         <is>
           <t>taux accises 1</t>
         </is>
       </c>
-      <c r="M1" t="n">
+      <c r="M1" s="0" t="n">
         <v>0.681339</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="0" t="inlineStr">
         <is>
           <t>Entrées</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="0" t="inlineStr">
         <is>
           <t>Sorties</t>
         </is>
@@ -57032,60 +57036,795 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="0" t="inlineStr">
         <is>
           <t>D&amp;B</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="0" t="inlineStr">
         <is>
           <t>R1152637567771</t>
         </is>
       </c>
-      <c r="C4" s="112" t="n">
+      <c r="C4" s="115" t="n">
         <v>46119</v>
       </c>
       <c r="D4" s="113" t="n">
         <v>55</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="F4" s="114" t="n">
+      <c r="F4" s="116" t="n">
         <v>37.473645</v>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="0" t="inlineStr">
         <is>
           <t>D&amp;B</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="0" t="inlineStr">
         <is>
           <t>D&amp;B</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="0" t="inlineStr">
         <is>
           <t>R1152637567771</t>
         </is>
       </c>
-      <c r="C5" s="112" t="n">
+      <c r="C5" s="115" t="n">
         <v>46119</v>
       </c>
       <c r="D5" s="113" t="n">
         <v>10</v>
       </c>
+      <c r="E5" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" s="116" t="n">
+        <v>11.92343</v>
+      </c>
+      <c r="G5" s="0" t="inlineStr">
+        <is>
+          <t>D&amp;B</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>Kirshner Fischer</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>RGK26-03163</t>
+        </is>
+      </c>
+      <c r="C6" s="115" t="n">
+        <v>46121</v>
+      </c>
+      <c r="D6" s="113" t="n">
+        <v>47</v>
+      </c>
+      <c r="E6" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="116" t="n">
+        <v>32.022933</v>
+      </c>
+      <c r="G6" s="0" t="inlineStr">
+        <is>
+          <t>Kirshner Fischer</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>Kirshner Fischer</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>RGK26-03222</t>
+        </is>
+      </c>
+      <c r="C7" s="115" t="n">
+        <v>46125</v>
+      </c>
+      <c r="D7" s="113" t="n">
+        <v>81</v>
+      </c>
+      <c r="E7" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="116" t="n">
+        <v>55.188459</v>
+      </c>
+      <c r="G7" s="0" t="inlineStr">
+        <is>
+          <t>Kirshner Fischer</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>Kirshner Fischer</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>RGK26-03223</t>
+        </is>
+      </c>
+      <c r="C8" s="115" t="n">
+        <v>46125</v>
+      </c>
+      <c r="D8" s="113" t="n">
+        <v>10</v>
+      </c>
+      <c r="E8" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="116" t="n">
+        <v>6.81339</v>
+      </c>
+      <c r="G8" s="0" t="inlineStr">
+        <is>
+          <t>Kirshner Fischer</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>Kirshner Fischer</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>RGK26-03268</t>
+        </is>
+      </c>
+      <c r="C9" s="115" t="n">
+        <v>46125</v>
+      </c>
+      <c r="D9" s="113" t="n">
+        <v>321</v>
+      </c>
+      <c r="E9" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="116" t="n">
+        <v>218.709819</v>
+      </c>
+      <c r="G9" s="0" t="inlineStr">
+        <is>
+          <t>Kirshner Fischer</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>Kirshner Fischer</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>RGK26-03333</t>
+        </is>
+      </c>
+      <c r="C10" s="115" t="n">
+        <v>46126</v>
+      </c>
+      <c r="D10" s="113" t="n">
+        <v>20</v>
+      </c>
+      <c r="E10" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="116" t="n">
+        <v>13.62678</v>
+      </c>
+      <c r="G10" s="0" t="inlineStr">
+        <is>
+          <t>Kirshner Fischer</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>Sinass</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>200295</t>
+        </is>
+      </c>
+      <c r="C11" s="115" t="n">
+        <v>46133</v>
+      </c>
+      <c r="D11" s="113" t="n">
+        <v>50</v>
+      </c>
+      <c r="E11" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="116" t="n">
+        <v>34.06695</v>
+      </c>
+      <c r="G11" s="0" t="inlineStr">
+        <is>
+          <t>Sinass</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>D&amp;B</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>R1154396567771</t>
+        </is>
+      </c>
+      <c r="C12" s="115" t="n">
+        <v>46134</v>
+      </c>
+      <c r="D12" s="113" t="n">
+        <v>20</v>
+      </c>
+      <c r="E12" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="116" t="n">
+        <v>13.62678</v>
+      </c>
+      <c r="G12" s="0" t="inlineStr">
+        <is>
+          <t>D&amp;B</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>D&amp;B</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>R1154396567771</t>
+        </is>
+      </c>
+      <c r="C13" s="115" t="n">
+        <v>46134</v>
+      </c>
+      <c r="D13" s="113" t="n">
+        <v>10</v>
+      </c>
+      <c r="E13" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="F13" s="116" t="n">
+        <v>11.92343</v>
+      </c>
+      <c r="G13" s="0" t="inlineStr">
+        <is>
+          <t>D&amp;B</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>Kirshner Fischer</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>RGK26-03604</t>
+        </is>
+      </c>
+      <c r="C14" s="115" t="n">
+        <v>46135</v>
+      </c>
+      <c r="D14" s="113" t="n">
+        <v>154.7</v>
+      </c>
+      <c r="E14" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="116" t="n">
+        <v>105.4031433</v>
+      </c>
+      <c r="G14" s="0" t="inlineStr">
+        <is>
+          <t>Kirshner Fischer</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>Kirshner Fischer</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>RGK26-03605</t>
+        </is>
+      </c>
+      <c r="C15" s="115" t="n">
+        <v>46135</v>
+      </c>
+      <c r="D15" s="113" t="n">
+        <v>92.87</v>
+      </c>
+      <c r="E15" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" s="116" t="n">
+        <v>63.27595293</v>
+      </c>
+      <c r="G15" s="0" t="inlineStr">
+        <is>
+          <t>Kirshner Fischer</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>Kirshner Fischer</t>
+        </is>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>RGK26-03606</t>
+        </is>
+      </c>
+      <c r="C16" s="115" t="n">
+        <v>46135</v>
+      </c>
+      <c r="D16" s="113" t="n">
+        <v>167.24</v>
+      </c>
+      <c r="E16" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="116" t="n">
+        <v>113.94713436</v>
+      </c>
+      <c r="G16" s="0" t="inlineStr">
+        <is>
+          <t>Kirshner Fischer</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>D&amp;B</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>R1155015567771</t>
+        </is>
+      </c>
+      <c r="C17" s="115" t="n">
+        <v>46139</v>
+      </c>
+      <c r="D17" s="113" t="n">
+        <v>25</v>
+      </c>
+      <c r="E17" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="F17" s="116" t="n">
+        <v>29.808575</v>
+      </c>
+      <c r="G17" s="0" t="inlineStr">
+        <is>
+          <t>D&amp;B</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>Kirshner Fischer</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>RGK26-03755</t>
+        </is>
+      </c>
+      <c r="C18" s="115" t="n">
+        <v>46139</v>
+      </c>
+      <c r="D18" s="113" t="n">
+        <v>20</v>
+      </c>
+      <c r="E18" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" s="116" t="n">
+        <v>13.62678</v>
+      </c>
+      <c r="G18" s="0" t="inlineStr">
+        <is>
+          <t>Kirshner Fischer</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>Kirshner Fischer</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>RGK26-03758</t>
+        </is>
+      </c>
+      <c r="C19" s="115" t="n">
+        <v>46139</v>
+      </c>
+      <c r="D19" s="113" t="n">
+        <v>10</v>
+      </c>
+      <c r="E19" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="116" t="n">
+        <v>6.81339</v>
+      </c>
+      <c r="G19" s="0" t="inlineStr">
+        <is>
+          <t>Kirshner Fischer</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>D&amp;B</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>R1155295567771</t>
+        </is>
+      </c>
+      <c r="C20" s="115" t="n">
+        <v>46140</v>
+      </c>
+      <c r="D20" s="113" t="n">
+        <v>26</v>
+      </c>
+      <c r="E20" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="F20" s="116" t="n">
+        <v>31.000918</v>
+      </c>
+      <c r="G20" s="0" t="inlineStr">
+        <is>
+          <t>D&amp;B</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>Kirshner Fischer</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>RGK26-03856</t>
+        </is>
+      </c>
+      <c r="C21" s="115" t="n">
+        <v>46142</v>
+      </c>
+      <c r="D21" s="113" t="n">
+        <v>20</v>
+      </c>
+      <c r="E21" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" s="116" t="n">
+        <v>13.62678</v>
+      </c>
+      <c r="G21" s="0" t="inlineStr">
+        <is>
+          <t>Kirshner Fischer</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>Sinass</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>200573</t>
+        </is>
+      </c>
+      <c r="C22" s="115" t="n">
+        <v>46142</v>
+      </c>
+      <c r="D22" s="113" t="n">
+        <v>110</v>
+      </c>
+      <c r="E22" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" s="116" t="n">
+        <v>74.94729000000001</v>
+      </c>
+      <c r="G22" s="0" t="inlineStr">
+        <is>
+          <t>Sinass</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>Total du mois</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="n">
+        <v>1249.81</v>
+      </c>
+      <c r="F23" s="0" t="n">
+        <v>887.8255795900002</v>
+      </c>
+      <c r="G23" s="0" t="inlineStr">
+        <is>
+          <t>Total du mois</t>
+        </is>
+      </c>
+      <c r="J23" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>Taux 1</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="n">
+        <v>1178.81</v>
+      </c>
+      <c r="F24" s="0" t="n">
+        <v>803.1692265900003</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>Taux 2</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="n">
+        <v>71</v>
+      </c>
+      <c r="F25" s="0" t="n">
+        <v>84.656353</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="D26" s="0" t="n">
+        <v>1249.81</v>
+      </c>
+      <c r="F26" s="0" t="n">
+        <v>887.8255795900003</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" style="104" min="1" max="1"/>
+    <col width="16" customWidth="1" style="104" min="2" max="2"/>
+    <col width="12" customWidth="1" style="104" min="3" max="3"/>
+    <col width="10" customWidth="1" style="104" min="4" max="4"/>
+    <col width="6" customWidth="1" style="104" min="5" max="5"/>
+    <col width="12" customWidth="1" style="104" min="6" max="6"/>
+    <col width="18" customWidth="1" style="104" min="7" max="7"/>
+    <col width="10" customWidth="1" style="104" min="8" max="8"/>
+    <col width="12" customWidth="1" style="104" min="9" max="9"/>
+    <col width="10" customWidth="1" style="104" min="10" max="10"/>
+    <col width="10" customWidth="1" style="104" min="11" max="11"/>
+    <col width="14" customWidth="1" style="104" min="12" max="12"/>
+    <col width="10" customWidth="1" style="104" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="111" t="inlineStr">
+        <is>
+          <t>Mai26</t>
+        </is>
+      </c>
+      <c r="G1" s="111" t="inlineStr">
+        <is>
+          <t>Mai26</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>taux accises 1</t>
+        </is>
+      </c>
+      <c r="M1" t="n">
+        <v>0.681339</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="111" t="inlineStr">
+        <is>
+          <t>Entrées</t>
+        </is>
+      </c>
+      <c r="G2" s="111" t="inlineStr">
+        <is>
+          <t>Sorties</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Fournisseurs</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Facture n°</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Kg de thé</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Taux</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Accises</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Fournisseurs</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>AC4 n°</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Kg de thé</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Accises</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Taux accises 2</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
+        <v>1.192343</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Kirshner Fischer</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>RGK26-04142</t>
+        </is>
+      </c>
+      <c r="C4" s="117" t="n">
+        <v>46153</v>
+      </c>
+      <c r="D4" t="n">
+        <v>40</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>27.25356</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Kirshner Fischer</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Kirshner Fischer</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>RGK26-04167</t>
+        </is>
+      </c>
+      <c r="C5" s="117" t="n">
+        <v>46154</v>
+      </c>
+      <c r="D5" t="n">
+        <v>30</v>
+      </c>
       <c r="E5" t="n">
-        <v>2</v>
-      </c>
-      <c r="F5" s="114" t="n">
-        <v>11.92343</v>
+        <v>1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>20.44017</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>D&amp;B</t>
+          <t>Kirshner Fischer</t>
         </is>
       </c>
     </row>
@@ -57097,20 +57836,20 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>RGK26-03163</t>
+          <t>RGK26-04188</t>
         </is>
       </c>
-      <c r="C6" s="112" t="n">
-        <v>46121</v>
-      </c>
-      <c r="D6" s="113" t="n">
-        <v>47</v>
+      <c r="C6" s="117" t="n">
+        <v>46154</v>
+      </c>
+      <c r="D6" t="n">
+        <v>40</v>
       </c>
       <c r="E6" t="n">
         <v>1</v>
       </c>
-      <c r="F6" s="114" t="n">
-        <v>32.022933</v>
+      <c r="F6" t="n">
+        <v>27.25356</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -57126,20 +57865,20 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>RGK26-03222</t>
+          <t>RGK26-04189</t>
         </is>
       </c>
-      <c r="C7" s="112" t="n">
-        <v>46125</v>
-      </c>
-      <c r="D7" s="113" t="n">
-        <v>81</v>
+      <c r="C7" s="117" t="n">
+        <v>46154</v>
+      </c>
+      <c r="D7" t="n">
+        <v>100</v>
       </c>
       <c r="E7" t="n">
         <v>1</v>
       </c>
-      <c r="F7" s="114" t="n">
-        <v>55.188459</v>
+      <c r="F7" t="n">
+        <v>68.1339</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -57155,20 +57894,20 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>RGK26-03223</t>
+          <t>RGK26-04267</t>
         </is>
       </c>
-      <c r="C8" s="112" t="n">
-        <v>46125</v>
-      </c>
-      <c r="D8" s="113" t="n">
-        <v>10</v>
+      <c r="C8" s="117" t="n">
+        <v>46160</v>
+      </c>
+      <c r="D8" t="n">
+        <v>170</v>
       </c>
       <c r="E8" t="n">
         <v>1</v>
       </c>
-      <c r="F8" s="114" t="n">
-        <v>6.81339</v>
+      <c r="F8" t="n">
+        <v>115.82763</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -57184,20 +57923,20 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>RGK26-03268</t>
+          <t>RGK26-04265</t>
         </is>
       </c>
-      <c r="C9" s="112" t="n">
-        <v>46125</v>
-      </c>
-      <c r="D9" s="113" t="n">
-        <v>321</v>
+      <c r="C9" s="117" t="n">
+        <v>46161</v>
+      </c>
+      <c r="D9" t="n">
+        <v>30</v>
       </c>
       <c r="E9" t="n">
         <v>1</v>
       </c>
-      <c r="F9" s="114" t="n">
-        <v>218.709819</v>
+      <c r="F9" t="n">
+        <v>20.44017</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -57213,20 +57952,20 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>RGK26-03333</t>
+          <t>RGK26-04266</t>
         </is>
       </c>
-      <c r="C10" s="112" t="n">
-        <v>46126</v>
-      </c>
-      <c r="D10" s="113" t="n">
-        <v>20</v>
+      <c r="C10" s="117" t="n">
+        <v>46161</v>
+      </c>
+      <c r="D10" t="n">
+        <v>49.7</v>
       </c>
       <c r="E10" t="n">
         <v>1</v>
       </c>
-      <c r="F10" s="114" t="n">
-        <v>13.62678</v>
+      <c r="F10" t="n">
+        <v>33.8625483</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -57237,58 +57976,58 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Sinass</t>
+          <t>Kirshner Fischer</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>200295</t>
+          <t>RGK26-04387</t>
         </is>
       </c>
-      <c r="C11" s="112" t="n">
-        <v>46133</v>
-      </c>
-      <c r="D11" s="113" t="n">
-        <v>50</v>
+      <c r="C11" s="117" t="n">
+        <v>46162</v>
+      </c>
+      <c r="D11" t="n">
+        <v>20</v>
       </c>
       <c r="E11" t="n">
         <v>1</v>
       </c>
-      <c r="F11" s="114" t="n">
-        <v>34.06695</v>
+      <c r="F11" t="n">
+        <v>13.62678</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Sinass</t>
+          <t>Kirshner Fischer</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>D&amp;B</t>
+          <t>Kirshner Fischer</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>R1154396567771</t>
+          <t>RGK26-04484</t>
         </is>
       </c>
-      <c r="C12" s="112" t="n">
-        <v>46134</v>
-      </c>
-      <c r="D12" s="113" t="n">
-        <v>20</v>
+      <c r="C12" s="117" t="n">
+        <v>46168</v>
+      </c>
+      <c r="D12" t="n">
+        <v>25</v>
       </c>
       <c r="E12" t="n">
         <v>1</v>
       </c>
-      <c r="F12" s="114" t="n">
-        <v>13.62678</v>
+      <c r="F12" t="n">
+        <v>17.033475</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>D&amp;B</t>
+          <t>Kirshner Fischer</t>
         </is>
       </c>
     </row>
@@ -57300,20 +58039,20 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>R1154396567771</t>
+          <t>R1159008567771</t>
         </is>
       </c>
-      <c r="C13" s="112" t="n">
-        <v>46134</v>
-      </c>
-      <c r="D13" s="113" t="n">
-        <v>10</v>
+      <c r="C13" s="117" t="n">
+        <v>46171</v>
+      </c>
+      <c r="D13" t="n">
+        <v>80</v>
       </c>
       <c r="E13" t="n">
-        <v>2</v>
-      </c>
-      <c r="F13" s="114" t="n">
-        <v>11.92343</v>
+        <v>1</v>
+      </c>
+      <c r="F13" t="n">
+        <v>54.50712</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -57324,320 +58063,98 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Kirshner Fischer</t>
+          <t>D&amp;B</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>RGK26-03604</t>
+          <t>R1159008567771</t>
         </is>
       </c>
-      <c r="C14" s="112" t="n">
-        <v>46135</v>
-      </c>
-      <c r="D14" s="113" t="n">
-        <v>154.7</v>
+      <c r="C14" s="117" t="n">
+        <v>46171</v>
+      </c>
+      <c r="D14" t="n">
+        <v>30</v>
       </c>
       <c r="E14" t="n">
-        <v>1</v>
-      </c>
-      <c r="F14" s="114" t="n">
-        <v>105.4031433</v>
+        <v>2</v>
+      </c>
+      <c r="F14" t="n">
+        <v>35.77029</v>
       </c>
       <c r="G14" t="inlineStr">
-        <is>
-          <t>Kirshner Fischer</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Kirshner Fischer</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>RGK26-03605</t>
-        </is>
-      </c>
-      <c r="C15" s="112" t="n">
-        <v>46135</v>
-      </c>
-      <c r="D15" s="113" t="n">
-        <v>92.87</v>
-      </c>
-      <c r="E15" t="n">
-        <v>1</v>
-      </c>
-      <c r="F15" s="114" t="n">
-        <v>63.27595293</v>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Kirshner Fischer</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Kirshner Fischer</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>RGK26-03606</t>
-        </is>
-      </c>
-      <c r="C16" s="112" t="n">
-        <v>46135</v>
-      </c>
-      <c r="D16" s="113" t="n">
-        <v>167.24</v>
-      </c>
-      <c r="E16" t="n">
-        <v>1</v>
-      </c>
-      <c r="F16" s="114" t="n">
-        <v>113.94713436</v>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Kirshner Fischer</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
         <is>
           <t>D&amp;B</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>R1155015567771</t>
-        </is>
-      </c>
-      <c r="C17" s="112" t="n">
-        <v>46139</v>
-      </c>
-      <c r="D17" s="113" t="n">
-        <v>25</v>
-      </c>
-      <c r="E17" t="n">
-        <v>2</v>
-      </c>
-      <c r="F17" s="114" t="n">
-        <v>29.808575</v>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>D&amp;B</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Kirshner Fischer</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>RGK26-03755</t>
-        </is>
-      </c>
-      <c r="C18" s="112" t="n">
-        <v>46139</v>
-      </c>
-      <c r="D18" s="113" t="n">
-        <v>20</v>
-      </c>
-      <c r="E18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F18" s="114" t="n">
-        <v>13.62678</v>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Kirshner Fischer</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Kirshner Fischer</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>RGK26-03758</t>
-        </is>
-      </c>
-      <c r="C19" s="112" t="n">
-        <v>46139</v>
-      </c>
-      <c r="D19" s="113" t="n">
-        <v>10</v>
-      </c>
-      <c r="E19" t="n">
-        <v>1</v>
-      </c>
-      <c r="F19" s="114" t="n">
-        <v>6.81339</v>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Kirshner Fischer</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>D&amp;B</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>R1155295567771</t>
-        </is>
-      </c>
-      <c r="C20" s="112" t="n">
-        <v>46140</v>
-      </c>
-      <c r="D20" s="113" t="n">
-        <v>26</v>
-      </c>
-      <c r="E20" t="n">
-        <v>2</v>
-      </c>
-      <c r="F20" s="114" t="n">
-        <v>31.000918</v>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>D&amp;B</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Kirshner Fischer</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>RGK26-03856</t>
-        </is>
-      </c>
-      <c r="C21" s="112" t="n">
-        <v>46142</v>
-      </c>
-      <c r="D21" s="113" t="n">
-        <v>20</v>
-      </c>
-      <c r="E21" t="n">
-        <v>1</v>
-      </c>
-      <c r="F21" s="114" t="n">
-        <v>13.62678</v>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Kirshner Fischer</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Sinass</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>200573</t>
-        </is>
-      </c>
-      <c r="C22" s="112" t="n">
-        <v>46142</v>
-      </c>
-      <c r="D22" s="113" t="n">
-        <v>110</v>
-      </c>
-      <c r="E22" t="n">
-        <v>1</v>
-      </c>
-      <c r="F22" s="114" t="n">
-        <v>74.94729000000001</v>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Sinass</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
+    </row>
+    <row r="15">
+      <c r="A15" s="111" t="inlineStr">
         <is>
           <t>Total du mois</t>
         </is>
       </c>
-      <c r="D23" t="n">
-        <v>1249.81</v>
-      </c>
-      <c r="F23" t="n">
-        <v>887.8255795900002</v>
-      </c>
-      <c r="G23" t="inlineStr">
+      <c r="D15">
+        <f>SUM(D4:D14)</f>
+        <v/>
+      </c>
+      <c r="F15">
+        <f>SUM(F4:F14)</f>
+        <v/>
+      </c>
+      <c r="G15" s="111" t="inlineStr">
         <is>
           <t>Total du mois</t>
         </is>
       </c>
-      <c r="J23" t="n">
-        <v>0</v>
-      </c>
-      <c r="K23" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="C24" t="inlineStr">
+      <c r="J15">
+        <f>SUM(J4:J14)</f>
+        <v/>
+      </c>
+      <c r="K15">
+        <f>SUM(K4:K14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="C16" t="inlineStr">
         <is>
           <t>Taux 1</t>
         </is>
       </c>
-      <c r="D24" t="n">
-        <v>1178.81</v>
-      </c>
-      <c r="F24" t="n">
-        <v>803.1692265900003</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="C25" t="inlineStr">
+      <c r="D16">
+        <f>SUMIF(E4:E14,1,D4:D14)</f>
+        <v/>
+      </c>
+      <c r="F16">
+        <f>SUMIF(E4:E14,1,F4:F14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="C17" t="inlineStr">
         <is>
           <t>Taux 2</t>
         </is>
       </c>
-      <c r="D25" t="n">
-        <v>71</v>
-      </c>
-      <c r="F25" t="n">
-        <v>84.656353</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="D26" t="n">
-        <v>1249.81</v>
-      </c>
-      <c r="F26" t="n">
-        <v>887.8255795900003</v>
+      <c r="D17">
+        <f>SUMIF(E4:E14,2,D4:D14)</f>
+        <v/>
+      </c>
+      <c r="F17">
+        <f>SUMIF(E4:E14,2,F4:F14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="D18">
+        <f>D16+D17</f>
+        <v/>
+      </c>
+      <c r="F18">
+        <f>F16+F17</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
accises: Mai-26 +2 factures KF debut mai (RGK26-03985 40kg, RGK26-03998 10kg) + onglet Annexe Mai26 P1 detail — total mois 664,7 kg / 468,22 EUR
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Accises/AC4_Tea_Tree_SA_Q126_updated v2.xlsx
+++ b/Accises/AC4_Tea_Tree_SA_Q126_updated v2.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q126" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Avril-26" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mai-26" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Annexe Mai26 P1" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -57655,7 +57656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M18"/>
+  <dimension ref="A1:M20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="104" min="1" max="1"/>
@@ -57778,11 +57779,11 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>RGK26-04142</t>
+          <t>RGK26-03985</t>
         </is>
       </c>
       <c r="C4" s="117" t="n">
-        <v>46153</v>
+        <v>46148</v>
       </c>
       <c r="D4" t="n">
         <v>40</v>
@@ -57807,20 +57808,20 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>RGK26-04167</t>
+          <t>RGK26-03998</t>
         </is>
       </c>
       <c r="C5" s="117" t="n">
-        <v>46154</v>
+        <v>46149</v>
       </c>
       <c r="D5" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E5" t="n">
         <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>20.44017</v>
+        <v>6.81339</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -57836,11 +57837,11 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>RGK26-04188</t>
+          <t>RGK26-04142</t>
         </is>
       </c>
       <c r="C6" s="117" t="n">
-        <v>46154</v>
+        <v>46153</v>
       </c>
       <c r="D6" t="n">
         <v>40</v>
@@ -57865,20 +57866,20 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>RGK26-04189</t>
+          <t>RGK26-04167</t>
         </is>
       </c>
       <c r="C7" s="117" t="n">
         <v>46154</v>
       </c>
       <c r="D7" t="n">
-        <v>100</v>
+        <v>30</v>
       </c>
       <c r="E7" t="n">
         <v>1</v>
       </c>
       <c r="F7" t="n">
-        <v>68.1339</v>
+        <v>20.44017</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -57894,20 +57895,20 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>RGK26-04267</t>
+          <t>RGK26-04188</t>
         </is>
       </c>
       <c r="C8" s="117" t="n">
-        <v>46160</v>
+        <v>46154</v>
       </c>
       <c r="D8" t="n">
-        <v>170</v>
+        <v>40</v>
       </c>
       <c r="E8" t="n">
         <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>115.82763</v>
+        <v>27.25356</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -57923,20 +57924,20 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>RGK26-04265</t>
+          <t>RGK26-04189</t>
         </is>
       </c>
       <c r="C9" s="117" t="n">
-        <v>46161</v>
+        <v>46154</v>
       </c>
       <c r="D9" t="n">
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="E9" t="n">
         <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>20.44017</v>
+        <v>68.1339</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -57952,20 +57953,20 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>RGK26-04266</t>
+          <t>RGK26-04267</t>
         </is>
       </c>
       <c r="C10" s="117" t="n">
-        <v>46161</v>
+        <v>46160</v>
       </c>
       <c r="D10" t="n">
-        <v>49.7</v>
+        <v>170</v>
       </c>
       <c r="E10" t="n">
         <v>1</v>
       </c>
       <c r="F10" t="n">
-        <v>33.8625483</v>
+        <v>115.82763</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -57981,20 +57982,20 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>RGK26-04387</t>
+          <t>RGK26-04265</t>
         </is>
       </c>
       <c r="C11" s="117" t="n">
-        <v>46162</v>
+        <v>46161</v>
       </c>
       <c r="D11" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="E11" t="n">
         <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>13.62678</v>
+        <v>20.44017</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -58010,20 +58011,20 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>RGK26-04484</t>
+          <t>RGK26-04266</t>
         </is>
       </c>
       <c r="C12" s="117" t="n">
-        <v>46168</v>
+        <v>46161</v>
       </c>
       <c r="D12" t="n">
-        <v>25</v>
+        <v>49.7</v>
       </c>
       <c r="E12" t="n">
         <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>17.033475</v>
+        <v>33.8625483</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -58034,127 +58035,915 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>D&amp;B</t>
+          <t>Kirshner Fischer</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>R1159008567771</t>
+          <t>RGK26-04387</t>
         </is>
       </c>
       <c r="C13" s="117" t="n">
-        <v>46171</v>
+        <v>46162</v>
       </c>
       <c r="D13" t="n">
-        <v>80</v>
+        <v>20</v>
       </c>
       <c r="E13" t="n">
         <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>54.50712</v>
+        <v>13.62678</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>D&amp;B</t>
+          <t>Kirshner Fischer</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>Kirshner Fischer</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>RGK26-04484</t>
+        </is>
+      </c>
+      <c r="C14" s="117" t="n">
+        <v>46168</v>
+      </c>
+      <c r="D14" t="n">
+        <v>25</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" t="n">
+        <v>17.033475</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Kirshner Fischer</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>D&amp;B</t>
         </is>
       </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>R1159008567771</t>
+        </is>
+      </c>
+      <c r="C15" s="117" t="n">
+        <v>46171</v>
+      </c>
+      <c r="D15" t="n">
+        <v>80</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" t="n">
+        <v>54.50712</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>D&amp;B</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>D&amp;B</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>R1159008567771</t>
+        </is>
+      </c>
+      <c r="C16" s="117" t="n">
+        <v>46171</v>
+      </c>
+      <c r="D16" t="n">
+        <v>30</v>
+      </c>
+      <c r="E16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F16" t="n">
+        <v>35.77029</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>D&amp;B</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="111" t="inlineStr">
+        <is>
+          <t>Total du mois</t>
+        </is>
+      </c>
+      <c r="D17">
+        <f>SUM(D4:D16)</f>
+        <v/>
+      </c>
+      <c r="F17">
+        <f>SUM(F4:F16)</f>
+        <v/>
+      </c>
+      <c r="G17" s="111" t="inlineStr">
+        <is>
+          <t>Total du mois</t>
+        </is>
+      </c>
+      <c r="J17">
+        <f>SUM(J4:J16)</f>
+        <v/>
+      </c>
+      <c r="K17">
+        <f>SUM(K4:K16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Taux 1</t>
+        </is>
+      </c>
+      <c r="D18">
+        <f>SUMIF(E4:E16,1,D4:D16)</f>
+        <v/>
+      </c>
+      <c r="F18">
+        <f>SUMIF(E4:E16,1,F4:F16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Taux 2</t>
+        </is>
+      </c>
+      <c r="D19">
+        <f>SUMIF(E4:E16,2,D4:D16)</f>
+        <v/>
+      </c>
+      <c r="F19">
+        <f>SUMIF(E4:E16,2,F4:F16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="D20">
+        <f>D18+D19</f>
+        <v/>
+      </c>
+      <c r="F20">
+        <f>F18+F19</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" style="104" min="1" max="1"/>
+    <col width="12" customWidth="1" style="104" min="2" max="2"/>
+    <col width="5" customWidth="1" style="104" min="3" max="3"/>
+    <col width="9" customWidth="1" style="104" min="4" max="4"/>
+    <col width="46" customWidth="1" style="104" min="5" max="5"/>
+    <col width="28" customWidth="1" style="104" min="6" max="6"/>
+    <col width="12" customWidth="1" style="104" min="7" max="7"/>
+    <col width="14" customWidth="1" style="104" min="8" max="8"/>
+    <col width="10" customWidth="1" style="104" min="9" max="9"/>
+    <col width="11" customWidth="1" style="104" min="10" max="10"/>
+    <col width="16" customWidth="1" style="104" min="11" max="11"/>
+    <col width="6" customWidth="1" style="104" min="12" max="12"/>
+    <col width="10" customWidth="1" style="104" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="111" t="inlineStr">
+        <is>
+          <t>ANNEXE DÉCLARATION ACCISES — Mai 2026 partie 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Tea Tree SA — Détail des factures RGK26-03985 et RGK26-03998 (Kirchner, Fischer &amp; Co GmbH)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="111" t="inlineStr">
+        <is>
+          <t>Facture n°</t>
+        </is>
+      </c>
+      <c r="B4" s="111" t="inlineStr">
+        <is>
+          <t>Date facture</t>
+        </is>
+      </c>
+      <c r="C4" s="111" t="inlineStr">
+        <is>
+          <t>Pos</t>
+        </is>
+      </c>
+      <c r="D4" s="111" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="E4" s="111" t="inlineStr">
+        <is>
+          <t>Description fournisseur</t>
+        </is>
+      </c>
+      <c r="F4" s="111" t="inlineStr">
+        <is>
+          <t>Réf. Teatower</t>
+        </is>
+      </c>
+      <c r="G4" s="111" t="inlineStr">
+        <is>
+          <t>Lot</t>
+        </is>
+      </c>
+      <c r="H4" s="111" t="inlineStr">
+        <is>
+          <t>Code tarifaire</t>
+        </is>
+      </c>
+      <c r="I4" s="111" t="inlineStr">
+        <is>
+          <t>Qté</t>
+        </is>
+      </c>
+      <c r="J4" s="111" t="inlineStr">
+        <is>
+          <t>Kg net thé</t>
+        </is>
+      </c>
+      <c r="K4" s="111" t="inlineStr">
+        <is>
+          <t>Soumis accises</t>
+        </is>
+      </c>
+      <c r="L4" s="111" t="inlineStr">
+        <is>
+          <t>Taux</t>
+        </is>
+      </c>
+      <c r="M4" s="111" t="inlineStr">
+        <is>
+          <t>Accises €</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>RGK26-03985</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>06/05/2026</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>36100</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Tea Ball Tong, stainless steel (Ø 4,5 cm)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>A0274 Filtre pince</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>LOTK046785</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>73239300900</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>3 × 24 pce</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Non — accessoire</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>RGK26-03985</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>06/05/2026</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>72046</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Teapot "Globe" verre 1500 ml</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>A0378 Théière en verre Wide</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>LOTK042637</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>70134200000</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>15 pce</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Non — accessoire</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>RGK26-03985</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>06/05/2026</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>26151</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Apple/Vanilla — flavoured fruit tea blend</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>MP_1V0257 Pomme vanille</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>LOTK066688</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>21069092859</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>5 × 1 kg</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>5</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="L7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M7" t="n">
+        <v>3.406695</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>RGK26-03985</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>06/05/2026</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>4</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>18804</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Fairy Dew — flavoured green tea</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>MP_1V0617 Liberté</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>LOTK070454</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>09021000000</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>10 × 1 kg</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>10</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="L8" t="n">
+        <v>1</v>
+      </c>
+      <c r="M8" t="n">
+        <v>6.81339</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>RGK26-03985</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>06/05/2026</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>5</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>18728</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>My Lady — flavoured black tea blend</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>MP_1V0772 Black Mango</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>LOTK068738</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>09023000000</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>10 × 1 kg</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>10</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="L9" t="n">
+        <v>1</v>
+      </c>
+      <c r="M9" t="n">
+        <v>6.81339</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>RGK26-03985</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>06/05/2026</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>6</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>18016</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Turkish Honey/White Nougat — flavoured black tea</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>18016</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>LOTK071198</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>09023000000</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>10 × 1 kg</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>10</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="L10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M10" t="n">
+        <v>6.81339</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>RGK26-03985</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>06/05/2026</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>7</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>25209</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Mocca/Cream — flavoured Rooibos blend</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>MP_1V0874 Café liégeois</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>LOTK065642</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>21069098690</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>5 × 1 kg</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>5</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="L11" t="n">
+        <v>1</v>
+      </c>
+      <c r="M11" t="n">
+        <v>3.406695</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>RGK26-03985</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>06/05/2026</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>8</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>1_VERS</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Assurance</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Non — frais</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>RGK26-03985</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>06/05/2026</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>9</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2_MAUT</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Péage</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Non — frais</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>RGK26-03998</t>
+        </is>
+      </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>R1159008567771</t>
-        </is>
-      </c>
-      <c r="C14" s="117" t="n">
-        <v>46171</v>
-      </c>
-      <c r="D14" t="n">
-        <v>30</v>
-      </c>
-      <c r="E14" t="n">
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>388124</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Fennel/Camomile — non-flavoured fruit/herbal tea blend</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>MP_1V0121 Lady Dodo</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>LOTK072410</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>21069092859</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>1 × 10 kg</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>10</v>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="L14" t="n">
+        <v>1</v>
+      </c>
+      <c r="M14" t="n">
+        <v>6.81339</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>RGK26-03998</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
         <v>2</v>
       </c>
-      <c r="F14" t="n">
-        <v>35.77029</v>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>D&amp;B</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="111" t="inlineStr">
-        <is>
-          <t>Total du mois</t>
-        </is>
-      </c>
-      <c r="D15">
-        <f>SUM(D4:D14)</f>
-        <v/>
-      </c>
-      <c r="F15">
-        <f>SUM(F4:F14)</f>
-        <v/>
-      </c>
-      <c r="G15" s="111" t="inlineStr">
-        <is>
-          <t>Total du mois</t>
-        </is>
-      </c>
-      <c r="J15">
-        <f>SUM(J4:J14)</f>
-        <v/>
-      </c>
-      <c r="K15">
-        <f>SUM(K4:K14)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Taux 1</t>
-        </is>
-      </c>
-      <c r="D16">
-        <f>SUMIF(E4:E14,1,D4:D14)</f>
-        <v/>
-      </c>
-      <c r="F16">
-        <f>SUMIF(E4:E14,1,F4:F14)</f>
-        <v/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2_MAUT</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Péage</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Non — frais</t>
+        </is>
       </c>
     </row>
     <row r="17">
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Taux 2</t>
-        </is>
-      </c>
-      <c r="D17">
-        <f>SUMIF(E4:E14,2,D4:D14)</f>
-        <v/>
-      </c>
-      <c r="F17">
-        <f>SUMIF(E4:E14,2,F4:F14)</f>
-        <v/>
+      <c r="A17" s="111" t="inlineStr">
+        <is>
+          <t>Sous-total RGK26-03985</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
+        <v>40</v>
+      </c>
+      <c r="L17" t="n">
+        <v>1</v>
+      </c>
+      <c r="M17" t="n">
+        <v>27.25356</v>
       </c>
     </row>
     <row r="18">
-      <c r="D18">
-        <f>D16+D17</f>
-        <v/>
-      </c>
-      <c r="F18">
-        <f>F16+F17</f>
-        <v/>
+      <c r="A18" s="111" t="inlineStr">
+        <is>
+          <t>Sous-total RGK26-03998</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>10</v>
+      </c>
+      <c r="L18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M18" t="n">
+        <v>6.81339</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="111" t="inlineStr">
+        <is>
+          <t>TOTAL partie 1</t>
+        </is>
+      </c>
+      <c r="J19" s="111" t="n">
+        <v>50</v>
+      </c>
+      <c r="M19" s="111" t="n">
+        <v>34.06695</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Taux accises 1 = 0.681339 €/kg (thé sans sucre ajouté) — Taux 2 = 1.192343 €/kg (avec sucre ajouté)</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
accises: declaration Mai26 partie 1 dans fichier SEPARE (AC4_Tea_Tree_SA_Mai26_partie1.xlsx, 50kg/34,07 EUR) - Mai-26 principal restaure a 614,7kg/434,15 EUR
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Accises/AC4_Tea_Tree_SA_Q126_updated v2.xlsx
+++ b/Accises/AC4_Tea_Tree_SA_Q126_updated v2.xlsx
@@ -11,7 +11,6 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q126" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Avril-26" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mai-26" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Annexe Mai26 P1" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -57656,7 +57655,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M20"/>
+  <dimension ref="A1:M18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="104" min="1" max="1"/>
@@ -57779,11 +57778,11 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>RGK26-03985</t>
+          <t>RGK26-04142</t>
         </is>
       </c>
       <c r="C4" s="117" t="n">
-        <v>46148</v>
+        <v>46153</v>
       </c>
       <c r="D4" t="n">
         <v>40</v>
@@ -57808,20 +57807,20 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>RGK26-03998</t>
+          <t>RGK26-04167</t>
         </is>
       </c>
       <c r="C5" s="117" t="n">
-        <v>46149</v>
+        <v>46154</v>
       </c>
       <c r="D5" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E5" t="n">
         <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>6.81339</v>
+        <v>20.44017</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -57837,11 +57836,11 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>RGK26-04142</t>
+          <t>RGK26-04188</t>
         </is>
       </c>
       <c r="C6" s="117" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="D6" t="n">
         <v>40</v>
@@ -57866,20 +57865,20 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>RGK26-04167</t>
+          <t>RGK26-04189</t>
         </is>
       </c>
       <c r="C7" s="117" t="n">
         <v>46154</v>
       </c>
       <c r="D7" t="n">
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="E7" t="n">
         <v>1</v>
       </c>
       <c r="F7" t="n">
-        <v>20.44017</v>
+        <v>68.1339</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -57895,20 +57894,20 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>RGK26-04188</t>
+          <t>RGK26-04267</t>
         </is>
       </c>
       <c r="C8" s="117" t="n">
-        <v>46154</v>
+        <v>46160</v>
       </c>
       <c r="D8" t="n">
-        <v>40</v>
+        <v>170</v>
       </c>
       <c r="E8" t="n">
         <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>27.25356</v>
+        <v>115.82763</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -57924,20 +57923,20 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>RGK26-04189</t>
+          <t>RGK26-04265</t>
         </is>
       </c>
       <c r="C9" s="117" t="n">
-        <v>46154</v>
+        <v>46161</v>
       </c>
       <c r="D9" t="n">
-        <v>100</v>
+        <v>30</v>
       </c>
       <c r="E9" t="n">
         <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>68.1339</v>
+        <v>20.44017</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -57953,20 +57952,20 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>RGK26-04267</t>
+          <t>RGK26-04266</t>
         </is>
       </c>
       <c r="C10" s="117" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="D10" t="n">
-        <v>170</v>
+        <v>49.7</v>
       </c>
       <c r="E10" t="n">
         <v>1</v>
       </c>
       <c r="F10" t="n">
-        <v>115.82763</v>
+        <v>33.8625483</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -57982,20 +57981,20 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>RGK26-04265</t>
+          <t>RGK26-04387</t>
         </is>
       </c>
       <c r="C11" s="117" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="D11" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="E11" t="n">
         <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>20.44017</v>
+        <v>13.62678</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -58011,20 +58010,20 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>RGK26-04266</t>
+          <t>RGK26-04484</t>
         </is>
       </c>
       <c r="C12" s="117" t="n">
-        <v>46161</v>
+        <v>46168</v>
       </c>
       <c r="D12" t="n">
-        <v>49.7</v>
+        <v>25</v>
       </c>
       <c r="E12" t="n">
         <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>33.8625483</v>
+        <v>17.033475</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -58035,915 +58034,127 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Kirshner Fischer</t>
+          <t>D&amp;B</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>RGK26-04387</t>
+          <t>R1159008567771</t>
         </is>
       </c>
       <c r="C13" s="117" t="n">
-        <v>46162</v>
+        <v>46171</v>
       </c>
       <c r="D13" t="n">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="E13" t="n">
         <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>13.62678</v>
+        <v>54.50712</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Kirshner Fischer</t>
+          <t>D&amp;B</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Kirshner Fischer</t>
+          <t>D&amp;B</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>RGK26-04484</t>
+          <t>R1159008567771</t>
         </is>
       </c>
       <c r="C14" s="117" t="n">
-        <v>46168</v>
+        <v>46171</v>
       </c>
       <c r="D14" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="E14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F14" t="n">
-        <v>17.033475</v>
+        <v>35.77029</v>
       </c>
       <c r="G14" t="inlineStr">
-        <is>
-          <t>Kirshner Fischer</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
         <is>
           <t>D&amp;B</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>R1159008567771</t>
-        </is>
-      </c>
-      <c r="C15" s="117" t="n">
-        <v>46171</v>
-      </c>
-      <c r="D15" t="n">
-        <v>80</v>
-      </c>
-      <c r="E15" t="n">
-        <v>1</v>
-      </c>
-      <c r="F15" t="n">
-        <v>54.50712</v>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>D&amp;B</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>D&amp;B</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>R1159008567771</t>
-        </is>
-      </c>
-      <c r="C16" s="117" t="n">
-        <v>46171</v>
-      </c>
-      <c r="D16" t="n">
-        <v>30</v>
-      </c>
-      <c r="E16" t="n">
-        <v>2</v>
-      </c>
-      <c r="F16" t="n">
-        <v>35.77029</v>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>D&amp;B</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="111" t="inlineStr">
+    </row>
+    <row r="15">
+      <c r="A15" s="111" t="inlineStr">
         <is>
           <t>Total du mois</t>
         </is>
       </c>
-      <c r="D17">
-        <f>SUM(D4:D16)</f>
+      <c r="D15">
+        <f>SUM(D4:D14)</f>
         <v/>
       </c>
-      <c r="F17">
-        <f>SUM(F4:F16)</f>
+      <c r="F15">
+        <f>SUM(F4:F14)</f>
         <v/>
       </c>
-      <c r="G17" s="111" t="inlineStr">
+      <c r="G15" s="111" t="inlineStr">
         <is>
           <t>Total du mois</t>
         </is>
       </c>
-      <c r="J17">
-        <f>SUM(J4:J16)</f>
+      <c r="J15">
+        <f>SUM(J4:J14)</f>
         <v/>
       </c>
-      <c r="K17">
-        <f>SUM(K4:K16)</f>
+      <c r="K15">
+        <f>SUM(K4:K14)</f>
         <v/>
       </c>
     </row>
-    <row r="18">
-      <c r="C18" t="inlineStr">
+    <row r="16">
+      <c r="C16" t="inlineStr">
         <is>
           <t>Taux 1</t>
         </is>
       </c>
-      <c r="D18">
-        <f>SUMIF(E4:E16,1,D4:D16)</f>
+      <c r="D16">
+        <f>SUMIF(E4:E14,1,D4:D14)</f>
         <v/>
       </c>
-      <c r="F18">
-        <f>SUMIF(E4:E16,1,F4:F16)</f>
+      <c r="F16">
+        <f>SUMIF(E4:E14,1,F4:F14)</f>
         <v/>
       </c>
     </row>
-    <row r="19">
-      <c r="C19" t="inlineStr">
+    <row r="17">
+      <c r="C17" t="inlineStr">
         <is>
           <t>Taux 2</t>
         </is>
       </c>
-      <c r="D19">
-        <f>SUMIF(E4:E16,2,D4:D16)</f>
+      <c r="D17">
+        <f>SUMIF(E4:E14,2,D4:D14)</f>
         <v/>
       </c>
-      <c r="F19">
-        <f>SUMIF(E4:E16,2,F4:F16)</f>
+      <c r="F17">
+        <f>SUMIF(E4:E14,2,F4:F14)</f>
         <v/>
       </c>
     </row>
-    <row r="20">
-      <c r="D20">
-        <f>D18+D19</f>
+    <row r="18">
+      <c r="D18">
+        <f>D16+D17</f>
         <v/>
       </c>
-      <c r="F20">
-        <f>F18+F19</f>
+      <c r="F18">
+        <f>F16+F17</f>
         <v/>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" style="104" min="1" max="1"/>
-    <col width="12" customWidth="1" style="104" min="2" max="2"/>
-    <col width="5" customWidth="1" style="104" min="3" max="3"/>
-    <col width="9" customWidth="1" style="104" min="4" max="4"/>
-    <col width="46" customWidth="1" style="104" min="5" max="5"/>
-    <col width="28" customWidth="1" style="104" min="6" max="6"/>
-    <col width="12" customWidth="1" style="104" min="7" max="7"/>
-    <col width="14" customWidth="1" style="104" min="8" max="8"/>
-    <col width="10" customWidth="1" style="104" min="9" max="9"/>
-    <col width="11" customWidth="1" style="104" min="10" max="10"/>
-    <col width="16" customWidth="1" style="104" min="11" max="11"/>
-    <col width="6" customWidth="1" style="104" min="12" max="12"/>
-    <col width="10" customWidth="1" style="104" min="13" max="13"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="111" t="inlineStr">
-        <is>
-          <t>ANNEXE DÉCLARATION ACCISES — Mai 2026 partie 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Tea Tree SA — Détail des factures RGK26-03985 et RGK26-03998 (Kirchner, Fischer &amp; Co GmbH)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="111" t="inlineStr">
-        <is>
-          <t>Facture n°</t>
-        </is>
-      </c>
-      <c r="B4" s="111" t="inlineStr">
-        <is>
-          <t>Date facture</t>
-        </is>
-      </c>
-      <c r="C4" s="111" t="inlineStr">
-        <is>
-          <t>Pos</t>
-        </is>
-      </c>
-      <c r="D4" s="111" t="inlineStr">
-        <is>
-          <t>Article</t>
-        </is>
-      </c>
-      <c r="E4" s="111" t="inlineStr">
-        <is>
-          <t>Description fournisseur</t>
-        </is>
-      </c>
-      <c r="F4" s="111" t="inlineStr">
-        <is>
-          <t>Réf. Teatower</t>
-        </is>
-      </c>
-      <c r="G4" s="111" t="inlineStr">
-        <is>
-          <t>Lot</t>
-        </is>
-      </c>
-      <c r="H4" s="111" t="inlineStr">
-        <is>
-          <t>Code tarifaire</t>
-        </is>
-      </c>
-      <c r="I4" s="111" t="inlineStr">
-        <is>
-          <t>Qté</t>
-        </is>
-      </c>
-      <c r="J4" s="111" t="inlineStr">
-        <is>
-          <t>Kg net thé</t>
-        </is>
-      </c>
-      <c r="K4" s="111" t="inlineStr">
-        <is>
-          <t>Soumis accises</t>
-        </is>
-      </c>
-      <c r="L4" s="111" t="inlineStr">
-        <is>
-          <t>Taux</t>
-        </is>
-      </c>
-      <c r="M4" s="111" t="inlineStr">
-        <is>
-          <t>Accises €</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>RGK26-03985</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>06/05/2026</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>36100</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Tea Ball Tong, stainless steel (Ø 4,5 cm)</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>A0274 Filtre pince</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>LOTK046785</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>73239300900</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>3 × 24 pce</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Non — accessoire</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>RGK26-03985</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>06/05/2026</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>72046</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Teapot "Globe" verre 1500 ml</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>A0378 Théière en verre Wide</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>LOTK042637</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>70134200000</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>15 pce</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Non — accessoire</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>RGK26-03985</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>06/05/2026</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>3</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>26151</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Apple/Vanilla — flavoured fruit tea blend</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>MP_1V0257 Pomme vanille</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>LOTK066688</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>21069092859</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>5 × 1 kg</t>
-        </is>
-      </c>
-      <c r="J7" t="n">
-        <v>5</v>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="L7" t="n">
-        <v>1</v>
-      </c>
-      <c r="M7" t="n">
-        <v>3.406695</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>RGK26-03985</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>06/05/2026</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>4</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>18804</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Fairy Dew — flavoured green tea</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>MP_1V0617 Liberté</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>LOTK070454</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>09021000000</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>10 × 1 kg</t>
-        </is>
-      </c>
-      <c r="J8" t="n">
-        <v>10</v>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="L8" t="n">
-        <v>1</v>
-      </c>
-      <c r="M8" t="n">
-        <v>6.81339</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>RGK26-03985</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>06/05/2026</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>5</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>18728</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>My Lady — flavoured black tea blend</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>MP_1V0772 Black Mango</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>LOTK068738</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>09023000000</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>10 × 1 kg</t>
-        </is>
-      </c>
-      <c r="J9" t="n">
-        <v>10</v>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="L9" t="n">
-        <v>1</v>
-      </c>
-      <c r="M9" t="n">
-        <v>6.81339</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>RGK26-03985</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>06/05/2026</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>6</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>18016</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Turkish Honey/White Nougat — flavoured black tea</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>18016</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>LOTK071198</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>09023000000</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>10 × 1 kg</t>
-        </is>
-      </c>
-      <c r="J10" t="n">
-        <v>10</v>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="L10" t="n">
-        <v>1</v>
-      </c>
-      <c r="M10" t="n">
-        <v>6.81339</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>RGK26-03985</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>06/05/2026</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>7</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>25209</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Mocca/Cream — flavoured Rooibos blend</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>MP_1V0874 Café liégeois</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>LOTK065642</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>21069098690</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>5 × 1 kg</t>
-        </is>
-      </c>
-      <c r="J11" t="n">
-        <v>5</v>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="L11" t="n">
-        <v>1</v>
-      </c>
-      <c r="M11" t="n">
-        <v>3.406695</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>RGK26-03985</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>06/05/2026</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>8</v>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>1_VERS</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Assurance</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>Non — frais</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>RGK26-03985</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>06/05/2026</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>9</v>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>2_MAUT</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Péage</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>Non — frais</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>RGK26-03998</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>388124</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Fennel/Camomile — non-flavoured fruit/herbal tea blend</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>MP_1V0121 Lady Dodo</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>LOTK072410</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>21069092859</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>1 × 10 kg</t>
-        </is>
-      </c>
-      <c r="J14" t="n">
-        <v>10</v>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="L14" t="n">
-        <v>1</v>
-      </c>
-      <c r="M14" t="n">
-        <v>6.81339</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>RGK26-03998</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>2</v>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>2_MAUT</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Péage</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>Non — frais</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="111" t="inlineStr">
-        <is>
-          <t>Sous-total RGK26-03985</t>
-        </is>
-      </c>
-      <c r="J17" t="n">
-        <v>40</v>
-      </c>
-      <c r="L17" t="n">
-        <v>1</v>
-      </c>
-      <c r="M17" t="n">
-        <v>27.25356</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="111" t="inlineStr">
-        <is>
-          <t>Sous-total RGK26-03998</t>
-        </is>
-      </c>
-      <c r="J18" t="n">
-        <v>10</v>
-      </c>
-      <c r="L18" t="n">
-        <v>1</v>
-      </c>
-      <c r="M18" t="n">
-        <v>6.81339</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="111" t="inlineStr">
-        <is>
-          <t>TOTAL partie 1</t>
-        </is>
-      </c>
-      <c r="J19" s="111" t="n">
-        <v>50</v>
-      </c>
-      <c r="M19" s="111" t="n">
-        <v>34.06695</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Taux accises 1 = 0.681339 €/kg (thé sans sucre ajouté) — Taux 2 = 1.192343 €/kg (avec sucre ajouté)</t>
-        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>